<commit_message>
Fix Balance Sheet to include Retained Earnings
- Add accumulated retained earnings tracking in batch_process_all_months.py
- Fix Income Statement to use period movements (not closing balances)
- Add Retained Earnings line to Equity section of Balance Sheet
- All 9 months (Feb-Oct 2025) now pass Module 7 validation
- Balance Sheet balances: Assets = Equity + Liabilities (Diff = 0.00)
- Generate audit_validation reports for all months

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/accountant-skill/data/output/Apr2025/financial_statements_Apr2025.xlsx
+++ b/accountant-skill/data/output/Apr2025/financial_statements_Apr2025.xlsx
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>103222000</v>
+        <v>52160000</v>
       </c>
     </row>
     <row r="6">
@@ -469,7 +469,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>92669732.17</v>
+        <v>45238168.11</v>
       </c>
     </row>
     <row r="7">
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>-195891732.17</v>
+        <v>6921831.890000001</v>
       </c>
     </row>
     <row r="9">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3758472.37</v>
+        <v>2306778.67</v>
       </c>
     </row>
     <row r="10">
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>-199650204.54</v>
+        <v>4615053.220000001</v>
       </c>
     </row>
     <row r="12">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>-199998234.54</v>
+        <v>4963083.220000001</v>
       </c>
     </row>
   </sheetData>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -716,23 +716,33 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Retained Earnings</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>5928126.530000004</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>TOTAL EQUITY</t>
         </is>
       </c>
-      <c r="B23" s="4" t="n">
-        <v>400000000</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="B24" s="4" t="n">
+        <v>405928126.53</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>TOTAL LIABILITIES &amp; EQUITY</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>400000000</v>
+      <c r="B26" s="4" t="n">
+        <v>405928126.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>